<commit_message>
Mise à jour des annonces — 2026-09-20 17:01
</commit_message>
<xml_diff>
--- a/annonces.xlsx
+++ b/annonces.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Annonces" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$293</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Annonces'!$A$1:$Q$292</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q293"/>
+  <dimension ref="A1:Q292"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -22408,17 +22408,17 @@
       </c>
       <c r="C254" s="6" t="inlineStr">
         <is>
-          <t>2 chambres meublé, secteur Place Valois (Hochelaga), près métro Joliette</t>
+          <t>6½ (3 chambres), rez-de-chaussée avec cour et stationnement - 27e Avenue (Rosemont, près métro D'Iberville)</t>
         </is>
       </c>
       <c r="D254" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E254" s="5" t="inlineStr">
         <is>
-          <t>2117A, Rue Nicolet, Montréal</t>
+          <t>6749, 27e Avenue, Montréal</t>
         </is>
       </c>
       <c r="F254" s="5" t="inlineStr">
@@ -22433,7 +22433,7 @@
       </c>
       <c r="H254" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I254" s="5" t="inlineStr">
@@ -22443,17 +22443,17 @@
       </c>
       <c r="J254" s="5" t="inlineStr">
         <is>
-          <t>Joliette</t>
+          <t>D'Iberville</t>
         </is>
       </c>
       <c r="K254" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>bleue</t>
         </is>
       </c>
       <c r="L254" s="5" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>1</t>
         </is>
       </c>
       <c r="M254" s="5" t="inlineStr">
@@ -22463,7 +22463,7 @@
       </c>
       <c r="N254" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-mercier-hochelaga-maisonneuve/21083818</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20987825</t>
         </is>
       </c>
       <c r="O254" s="5" t="inlineStr">
@@ -22473,12 +22473,12 @@
       </c>
       <c r="P254" s="6" t="inlineStr">
         <is>
-          <t>Meublé et équipé (laveuse-sécheuse, frigo, cuisinière, lave-vaisselle inclus), internet inclus, secteur Place Valois, Walk Score 97, disponible 7 jours après acceptation, superficie et balcon non précisés</t>
+          <t>7 pièces, rez-de-chaussée de triplex avec sous-sol, cour et stationnement inclus, animaux permis sur analyse, disponible 1er juillet 2026, métro Fabre aussi accessible (~5 min)</t>
         </is>
       </c>
       <c r="Q254" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15AD50DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6C9AB9DDDDDDDDDDC&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -22495,22 +22495,22 @@
       </c>
       <c r="C255" s="6" t="inlineStr">
         <is>
-          <t>6½ (3 chambres), rez-de-chaussée avec cour et stationnement - 27e Avenue (Rosemont, près métro D'Iberville)</t>
+          <t>5½ semi-meublé, 3 grandes chambres - rue Saint-Hubert (Villeray, près métro Jarry)</t>
         </is>
       </c>
       <c r="D255" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E255" s="5" t="inlineStr">
         <is>
-          <t>6749, 27e Avenue, Montréal</t>
+          <t>7635, Rue Saint-Hubert, Montréal</t>
         </is>
       </c>
       <c r="F255" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="G255" s="5" t="inlineStr">
@@ -22530,17 +22530,17 @@
       </c>
       <c r="J255" s="5" t="inlineStr">
         <is>
-          <t>D'Iberville</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K255" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L255" s="5" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M255" s="5" t="inlineStr">
@@ -22550,7 +22550,7 @@
       </c>
       <c r="N255" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20987825</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/25817021</t>
         </is>
       </c>
       <c r="O255" s="5" t="inlineStr">
@@ -22560,19 +22560,19 @@
       </c>
       <c r="P255" s="6" t="inlineStr">
         <is>
-          <t>7 pièces, rez-de-chaussée de triplex avec sous-sol, cour et stationnement inclus, animaux permis sur analyse, disponible 1er juillet 2026, métro Fabre aussi accessible (~5 min)</t>
+          <t>Semi-meublé, animaux acceptés sous conditions, disponible 1er juillet 2026, à ~11 min du métro Jarry (proche de la limite de 12 min) ; à ne pas confondre avec le 7639 rue Saint-Hubert déjà répertorié (adresse voisine, annonce distincte)</t>
         </is>
       </c>
       <c r="Q255" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6C9AB9DDDDDDDDDDC&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD627F1DDDDDDDDDD2&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="256">
       <c r="A256" s="5" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B256" s="5" t="inlineStr">
@@ -22582,22 +22582,22 @@
       </c>
       <c r="C256" s="6" t="inlineStr">
         <is>
-          <t>5½ semi-meublé, 3 grandes chambres - rue Saint-Hubert (Villeray, près métro Jarry)</t>
+          <t>4 chambres meublé, Plateau-Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D256" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E256" s="5" t="inlineStr">
         <is>
-          <t>7635, Rue Saint-Hubert, Montréal</t>
+          <t>3681, avenue Coloniale, Montréal (H2X 2Y7)</t>
         </is>
       </c>
       <c r="F256" s="5" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G256" s="5" t="inlineStr">
@@ -22607,7 +22607,7 @@
       </c>
       <c r="H256" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I256" s="5" t="inlineStr">
@@ -22617,7 +22617,7 @@
       </c>
       <c r="J256" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Mont-Royal ou Sherbrooke (à vérifier)</t>
         </is>
       </c>
       <c r="K256" s="5" t="inlineStr">
@@ -22627,17 +22627,17 @@
       </c>
       <c r="L256" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M256" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N256" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-villeray-saint-michel-parc-extension/25817021</t>
+          <t>https://www.facebook.com/marketplace/item/1578661203923320</t>
         </is>
       </c>
       <c r="O256" s="5" t="inlineStr">
@@ -22647,19 +22647,19 @@
       </c>
       <c r="P256" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, animaux acceptés sous conditions, disponible 1er juillet 2026, à ~11 min du métro Jarry (proche de la limite de 12 min) ; à ne pas confondre avec le 7639 rue Saint-Hubert déjà répertorié (adresse voisine, annonce distincte)</t>
+          <t>Meublé, orienté étudiants, bail 1 an, dispo maintenant. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q256" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD627F1DDDDDDDDDD2&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/746058480_2385279625296639_1965210297754561149_n.jpg?stp=c93.0.895.895a_dst-jpg_tt6&amp;cstp=mx895x895&amp;ctp=s565x565&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=ngElLDKbnLQQ7kNvwHndFuc&amp;_nc_oc=AdpOYEcvWwImdnqaiYyy1pwfVcV2sab1mFRQ5KYGa5FE_CkYORsBa8yvv6PCL2lbQ7E&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=EorVHkPe0HNRZxtO75C5fg&amp;_nc_ss=7f2a8&amp;oh=00_AQBlE2b8WT_3jlX6ddiFysYujtaCjsMiZRfF96JJT7pp3g&amp;oe=6A60805A</t>
         </is>
       </c>
     </row>
     <row r="257">
       <c r="A257" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B257" s="5" t="inlineStr">
@@ -22669,17 +22669,17 @@
       </c>
       <c r="C257" s="6" t="inlineStr">
         <is>
-          <t>4 chambres meublé, Plateau-Mont-Royal (Marketplace)</t>
+          <t>4½ moderne, thermopompe - avenue Papineau (Centre-Sud)</t>
         </is>
       </c>
       <c r="D257" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Ville-Marie (Centre-Sud)</t>
         </is>
       </c>
       <c r="E257" s="5" t="inlineStr">
         <is>
-          <t>3681, avenue Coloniale, Montréal (H2X 2Y7)</t>
+          <t>2121 Avenue Papineau, app. 106, Montréal</t>
         </is>
       </c>
       <c r="F257" s="5" t="inlineStr">
@@ -22694,59 +22694,59 @@
       </c>
       <c r="H257" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I257" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J257" s="5" t="inlineStr">
+        <is>
+          <t>Papineau</t>
+        </is>
+      </c>
+      <c r="K257" s="5" t="inlineStr">
+        <is>
+          <t>verte</t>
+        </is>
+      </c>
+      <c r="L257" s="5" t="inlineStr">
+        <is>
+          <t>11 (estimé)</t>
+        </is>
+      </c>
+      <c r="M257" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="N257" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1345509854217640</t>
+        </is>
+      </c>
+      <c r="O257" s="5" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I257" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J257" s="5" t="inlineStr">
-        <is>
-          <t>Mont-Royal ou Sherbrooke (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K257" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L257" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M257" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N257" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1578661203923320</t>
-        </is>
-      </c>
-      <c r="O257" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P257" s="6" t="inlineStr">
         <is>
-          <t>Meublé, orienté étudiants, bail 1 an, dispo maintenant. Lien Facebook (connexion requise)</t>
+          <t>Thermopompe (chauffage/climatisation), 5 électros inclus, stationnement intérieur +200$/mois, dispo 1er sept 2026. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q257" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/746058480_2385279625296639_1965210297754561149_n.jpg?stp=c93.0.895.895a_dst-jpg_tt6&amp;cstp=mx895x895&amp;ctp=s565x565&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=ngElLDKbnLQQ7kNvwHndFuc&amp;_nc_oc=AdpOYEcvWwImdnqaiYyy1pwfVcV2sab1mFRQ5KYGa5FE_CkYORsBa8yvv6PCL2lbQ7E&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=EorVHkPe0HNRZxtO75C5fg&amp;_nc_ss=7f2a8&amp;oh=00_AQBlE2b8WT_3jlX6ddiFysYujtaCjsMiZRfF96JJT7pp3g&amp;oe=6A60805A</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/740967146_10163353758868282_6445879430357129287_n.jpg?stp=c267.0.1067.1067a_dst-jpg_tt6&amp;cstp=mx1067x1067&amp;ctp=s565x565&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=NBpCPM0lMZ0Q7kNvwEgcjRv&amp;_nc_oc=AdpKpJOW9gIXzADTI6MMd8QgF1AIUSvmXyA1OhFaypIfCHhp5Q_WLet_FlJK9JeWopU&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=po_Fub79cNJDfbGc2ZS1tQ&amp;_nc_ss=7f2a8&amp;oh=00_AQAYyDy-ZzVKaSsRH6KHfK-C3t6CRRIgCb8d-ae59ygZwA&amp;oe=6A5E8565</t>
         </is>
       </c>
     </row>
     <row r="258">
       <c r="A258" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B258" s="5" t="inlineStr">
@@ -22756,22 +22756,22 @@
       </c>
       <c r="C258" s="6" t="inlineStr">
         <is>
-          <t>4½ moderne, thermopompe - avenue Papineau (Centre-Sud)</t>
+          <t>Grand 4 chambres + bureau – St-André bas Plateau</t>
         </is>
       </c>
       <c r="D258" s="5" t="inlineStr">
         <is>
-          <t>Ville-Marie (Centre-Sud)</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E258" s="5" t="inlineStr">
         <is>
-          <t>2121 Avenue Papineau, app. 106, Montréal</t>
+          <t>3855 rue St-André (H2L 3V9)</t>
         </is>
       </c>
       <c r="F258" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2395</t>
         </is>
       </c>
       <c r="G258" s="5" t="inlineStr">
@@ -22781,7 +22781,7 @@
       </c>
       <c r="H258" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>4</t>
         </is>
       </c>
       <c r="I258" s="5" t="inlineStr">
@@ -22791,17 +22791,17 @@
       </c>
       <c r="J258" s="5" t="inlineStr">
         <is>
-          <t>Papineau</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K258" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L258" s="5" t="inlineStr">
         <is>
-          <t>11 (estimé)</t>
+          <t>7</t>
         </is>
       </c>
       <c r="M258" s="5" t="inlineStr">
@@ -22811,7 +22811,7 @@
       </c>
       <c r="N258" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1345509854217640</t>
+          <t>https://www.facebook.com/marketplace/item/1550150270173512</t>
         </is>
       </c>
       <c r="O258" s="5" t="inlineStr">
@@ -22821,19 +22821,19 @@
       </c>
       <c r="P258" s="6" t="inlineStr">
         <is>
-          <t>Thermopompe (chauffage/climatisation), 5 électros inclus, stationnement intérieur +200$/mois, dispo 1er sept 2026. Lien Facebook (connexion requise)</t>
+          <t>4 chambres (dont 1 sans fenêtre) + bureau fermé, électros inclus, dispo 1er juillet. ~7 min à pied du métro Sherbrooke (estimé depuis l'adresse). Superficie non indiquée. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q258" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/740967146_10163353758868282_6445879430357129287_n.jpg?stp=c267.0.1067.1067a_dst-jpg_tt6&amp;cstp=mx1067x1067&amp;ctp=s565x565&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=NBpCPM0lMZ0Q7kNvwEgcjRv&amp;_nc_oc=AdpKpJOW9gIXzADTI6MMd8QgF1AIUSvmXyA1OhFaypIfCHhp5Q_WLet_FlJK9JeWopU&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=po_Fub79cNJDfbGc2ZS1tQ&amp;_nc_ss=7f2a8&amp;oh=00_AQAYyDy-ZzVKaSsRH6KHfK-C3t6CRRIgCb8d-ae59ygZwA&amp;oe=6A5E8565</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/728474326_10231683771185831_6727292866936668830_n.jpg?stp=c256.0.1537.1537a_dst-jpg_tt6&amp;cstp=mx1537x1537&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=943KDXUX1RQQ7kNvwFf3aXH&amp;_nc_oc=AdqiIy58nJFG1aGG5u9HQW6_QOL-2IMomb6kZpX5RbtE63MiJU-sRJMxj6FOz1Mq-C8&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=fqv6VHej6TNF8DZvOf_nSw&amp;_nc_ss=7f2a8&amp;oh=00_AQDIA5orKA1mjUQENX8o5T3X6Cteocg2jKTYaTNLxvUcJw&amp;oe=6A5D72DF</t>
         </is>
       </c>
     </row>
     <row r="259">
       <c r="A259" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B259" s="5" t="inlineStr">
@@ -22843,7 +22843,7 @@
       </c>
       <c r="C259" s="6" t="inlineStr">
         <is>
-          <t>Grand 4 chambres + bureau – St-André bas Plateau</t>
+          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
         </is>
       </c>
       <c r="D259" s="5" t="inlineStr">
@@ -22853,12 +22853,12 @@
       </c>
       <c r="E259" s="5" t="inlineStr">
         <is>
-          <t>3855 rue St-André (H2L 3V9)</t>
+          <t>4275 Rue de Bordeaux, Montréal</t>
         </is>
       </c>
       <c r="F259" s="5" t="inlineStr">
         <is>
-          <t>2395</t>
+          <t>2095</t>
         </is>
       </c>
       <c r="G259" s="5" t="inlineStr">
@@ -22868,59 +22868,59 @@
       </c>
       <c r="H259" s="5" t="inlineStr">
         <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I259" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J259" s="5" t="inlineStr">
+        <is>
+          <t>Mont-Royal</t>
+        </is>
+      </c>
+      <c r="K259" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L259" s="5" t="inlineStr">
+        <is>
+          <t>10 (estimé)</t>
+        </is>
+      </c>
+      <c r="M259" s="5" t="inlineStr">
+        <is>
+          <t>DuProprio</t>
+        </is>
+      </c>
+      <c r="N259" s="7" t="inlineStr">
+        <is>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+        </is>
+      </c>
+      <c r="O259" s="5" t="inlineStr">
+        <is>
           <t>4</t>
         </is>
       </c>
-      <c r="I259" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J259" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke</t>
-        </is>
-      </c>
-      <c r="K259" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L259" s="5" t="inlineStr">
-        <is>
-          <t>7</t>
-        </is>
-      </c>
-      <c r="M259" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N259" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1550150270173512</t>
-        </is>
-      </c>
-      <c r="O259" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P259" s="6" t="inlineStr">
         <is>
-          <t>4 chambres (dont 1 sans fenêtre) + bureau fermé, électros inclus, dispo 1er juillet. ~7 min à pied du métro Sherbrooke (estimé depuis l'adresse). Superficie non indiquée. Lien Facebook (connexion requise)</t>
+          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
         </is>
       </c>
       <c r="Q259" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/728474326_10231683771185831_6727292866936668830_n.jpg?stp=c256.0.1537.1537a_dst-jpg_tt6&amp;cstp=mx1537x1537&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=943KDXUX1RQQ7kNvwFf3aXH&amp;_nc_oc=AdqiIy58nJFG1aGG5u9HQW6_QOL-2IMomb6kZpX5RbtE63MiJU-sRJMxj6FOz1Mq-C8&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=fqv6VHej6TNF8DZvOf_nSw&amp;_nc_ss=7f2a8&amp;oh=00_AQDIA5orKA1mjUQENX8o5T3X6Cteocg2jKTYaTNLxvUcJw&amp;oe=6A5D72DF</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
         </is>
       </c>
     </row>
     <row r="260">
       <c r="A260" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B260" s="5" t="inlineStr">
@@ -22930,7 +22930,7 @@
       </c>
       <c r="C260" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres, près métro Mont-Royal (rue de Bordeaux)</t>
+          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
         </is>
       </c>
       <c r="D260" s="5" t="inlineStr">
@@ -22940,12 +22940,12 @@
       </c>
       <c r="E260" s="5" t="inlineStr">
         <is>
-          <t>4275 Rue de Bordeaux, Montréal</t>
+          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
         </is>
       </c>
       <c r="F260" s="5" t="inlineStr">
         <is>
-          <t>2095</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G260" s="5" t="inlineStr">
@@ -22965,7 +22965,7 @@
       </c>
       <c r="J260" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Mont-Royal ou Papineau (à vérifier)</t>
         </is>
       </c>
       <c r="K260" s="5" t="inlineStr">
@@ -22975,7 +22975,7 @@
       </c>
       <c r="L260" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>12 (estimé)</t>
         </is>
       </c>
       <c r="M260" s="5" t="inlineStr">
@@ -22985,7 +22985,7 @@
       </c>
       <c r="N260" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-4275-bordeaux-1131937</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
         </is>
       </c>
       <c r="O260" s="5" t="inlineStr">
@@ -22995,19 +22995,19 @@
       </c>
       <c r="P260" s="6" t="inlineStr">
         <is>
-          <t>2e étage, dispo immédiatement, rien d'inclus (chauffage/électricité aux frais du locataire), à moins de 10 min du parc La Fontaine, proche avenue du Mont-Royal (commerces/cafés), balcon et superficie non précisés dans l'annonce</t>
+          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
         </is>
       </c>
       <c r="Q260" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1131937/plateau-mont-royal-600-15652873.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
         </is>
       </c>
     </row>
     <row r="261">
       <c r="A261" s="5" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B261" s="5" t="inlineStr">
@@ -23017,7 +23017,7 @@
       </c>
       <c r="C261" s="6" t="inlineStr">
         <is>
-          <t>5 1/2, 3 chambres – Plateau (avenue de Lorimier)</t>
+          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
         </is>
       </c>
       <c r="D261" s="5" t="inlineStr">
@@ -23027,12 +23027,12 @@
       </c>
       <c r="E261" s="5" t="inlineStr">
         <is>
-          <t>4216 avenue de Lorimier, app. 204, Montréal</t>
+          <t>62 rue Rachel Est, Montréal</t>
         </is>
       </c>
       <c r="F261" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2195</t>
         </is>
       </c>
       <c r="G261" s="5" t="inlineStr">
@@ -23052,7 +23052,7 @@
       </c>
       <c r="J261" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal ou Papineau (à vérifier)</t>
+          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
         </is>
       </c>
       <c r="K261" s="5" t="inlineStr">
@@ -23062,7 +23062,7 @@
       </c>
       <c r="L261" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M261" s="5" t="inlineStr">
@@ -23072,7 +23072,7 @@
       </c>
       <c r="N261" s="7" t="inlineStr">
         <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-204-4216-av-de-lorimier-1135328</t>
+          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
         </is>
       </c>
       <c r="O261" s="5" t="inlineStr">
@@ -23082,19 +23082,19 @@
       </c>
       <c r="P261" s="6" t="inlineStr">
         <is>
-          <t>Semi-meublé, laveuse-sécheuse/cuisinière/frigo inclus, wifi inclus, 2e étage, petits animaux acceptés, dispo 1er juillet ou 1er sept 2026, balcon non précisé dans l'annonce, secteur commerçant (cafés, parcs) à pied</t>
+          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
         </is>
       </c>
       <c r="Q261" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202606/1135328/5-1-2-plateau-mont-royal-600-15736059.jpg</t>
+          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
         </is>
       </c>
     </row>
     <row r="262">
       <c r="A262" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B262" s="5" t="inlineStr">
@@ -23104,22 +23104,22 @@
       </c>
       <c r="C262" s="6" t="inlineStr">
         <is>
-          <t>Grand 5 1/2, 3 chambres fermées – coeur du Plateau (rue Rachel Est)</t>
+          <t>5½ rénové - Rosemont, 3 chambres + bureau (Marketplace)</t>
         </is>
       </c>
       <c r="D262" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E262" s="5" t="inlineStr">
         <is>
-          <t>62 rue Rachel Est, Montréal</t>
+          <t>n/d (secteur Rosemont, Montréal)</t>
         </is>
       </c>
       <c r="F262" s="5" t="inlineStr">
         <is>
-          <t>2195</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G262" s="5" t="inlineStr">
@@ -23129,59 +23129,59 @@
       </c>
       <c r="H262" s="5" t="inlineStr">
         <is>
+          <t>3 (selon titre, à confirmer)</t>
+        </is>
+      </c>
+      <c r="I262" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J262" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K262" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L262" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M262" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="N262" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1905640337262053</t>
+        </is>
+      </c>
+      <c r="O262" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I262" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J262" s="5" t="inlineStr">
-        <is>
-          <t>Sherbrooke ou Mont-Royal (à vérifier)</t>
-        </is>
-      </c>
-      <c r="K262" s="5" t="inlineStr">
-        <is>
-          <t>orange</t>
-        </is>
-      </c>
-      <c r="L262" s="5" t="inlineStr">
-        <is>
-          <t>8 (estimé)</t>
-        </is>
-      </c>
-      <c r="M262" s="5" t="inlineStr">
-        <is>
-          <t>DuProprio</t>
-        </is>
-      </c>
-      <c r="N262" s="7" t="inlineStr">
-        <is>
-          <t>https://duproprio.com/fr/location/montreal/le-plateau-mont-royal/5-1-2-a-louer/hab-5-12-62-rue-rachel-est-1132358</t>
-        </is>
-      </c>
-      <c r="O262" s="5" t="inlineStr">
-        <is>
-          <t>4</t>
-        </is>
-      </c>
       <c r="P262" s="6" t="inlineStr">
         <is>
-          <t>Dernier étage, tranquille et lumineux, entrée laveuse-sécheuse, non-fumeur, chiens non acceptés, enquête de crédit requise, balcon et superficie non précisés dans l'annonce, secteur près Saint-Laurent/Saint-Denis</t>
+          <t>Annonce titre seulement (« 5 1/2 rénové - Rosemont - 3 chambres + bureau »), aucune adresse ni description détaillée disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q262" s="5" t="inlineStr">
         <is>
-          <t>https://photos.duproprio.com/photos/public/for_rent/202605/1132358/5-1-2-plateau-mont-royal-1600-15661700.jpg</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/787761292_1065504692896878_4836055761486525916_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=MOCJ79afpPoQ7kNvwHB1OUw&amp;_nc_oc=Adr_kZR22WI-TaE-t3PMKjYftS_SVUX2bAUlPv8Qz_8bghKNDkoSXa2JK6t9RqxndLc&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=wgjL71BuqJilZmCDsgzwAw&amp;_nc_ss=7f289&amp;oh=00_AQIu4EnP-eitSmW9cB7PzqKfHZ07AHdQlQEc8LQQHjmjMA&amp;oe=6A9DD845</t>
         </is>
       </c>
     </row>
     <row r="263">
       <c r="A263" s="5" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B263" s="5" t="inlineStr">
@@ -23191,7 +23191,7 @@
       </c>
       <c r="C263" s="6" t="inlineStr">
         <is>
-          <t>5½ rénové - Rosemont, 3 chambres + bureau (Marketplace)</t>
+          <t>Logement 5 1/2 rénové, 3 chambres + bureau - Rosemont (Marketplace)</t>
         </is>
       </c>
       <c r="D263" s="5" t="inlineStr">
@@ -23201,7 +23201,7 @@
       </c>
       <c r="E263" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Rosemont, Montréal)</t>
+          <t>n/d (secteur Rosemont-La Petite-Patrie, Montréal)</t>
         </is>
       </c>
       <c r="F263" s="5" t="inlineStr">
@@ -23216,7 +23216,7 @@
       </c>
       <c r="H263" s="5" t="inlineStr">
         <is>
-          <t>3 (selon titre, à confirmer)</t>
+          <t>3 (estimé)</t>
         </is>
       </c>
       <c r="I263" s="5" t="inlineStr">
@@ -23246,7 +23246,7 @@
       </c>
       <c r="N263" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1905640337262053</t>
+          <t>https://www.facebook.com/marketplace/item/1613584236892605</t>
         </is>
       </c>
       <c r="O263" s="5" t="inlineStr">
@@ -23256,19 +23256,19 @@
       </c>
       <c r="P263" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (« 5 1/2 rénové - Rosemont - 3 chambres + bureau »), aucune adresse ni description détaillée disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Annonce titre seulement (« Logement 5 1/2 rénové Rosemont - 3 chambres + bureau »), aucune adresse ni description détaillée disponible via le scraper. Nombre de chambres selon le titre (3 + bureau). Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q263" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/787761292_1065504692896878_4836055761486525916_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=MOCJ79afpPoQ7kNvwHB1OUw&amp;_nc_oc=Adr_kZR22WI-TaE-t3PMKjYftS_SVUX2bAUlPv8Qz_8bghKNDkoSXa2JK6t9RqxndLc&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=wgjL71BuqJilZmCDsgzwAw&amp;_nc_ss=7f289&amp;oh=00_AQIu4EnP-eitSmW9cB7PzqKfHZ07AHdQlQEc8LQQHjmjMA&amp;oe=6A9DD845</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/789845450_1602489944997832_5213134105176151966_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xzqo9iyYcAkQ7kNvwHRvmWj&amp;_nc_oc=Adp04UM8mMS7TYZztbruBwtONw22BOWfpCFSRMezlhO7JaSrV4L2CIIxMvRmLg4IrzQ&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=iDnTU3IQw0eGZCC-IJSGrw&amp;_nc_ss=7f2a8&amp;oh=00_AQKWwqFPn5wiyRr8UhOqIiE2fW-83zbjH04dhSzspmsjgw&amp;oe=6A9A671F</t>
         </is>
       </c>
     </row>
     <row r="264">
       <c r="A264" s="5" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B264" s="5" t="inlineStr">
@@ -23278,7 +23278,7 @@
       </c>
       <c r="C264" s="6" t="inlineStr">
         <is>
-          <t>Logement 5 1/2 rénové, 3 chambres + bureau - Rosemont (Marketplace)</t>
+          <t>4½ rénové (2 chambres), semi-meublé - Plaza St-Hubert (Rosemont), près du métro Beaubien</t>
         </is>
       </c>
       <c r="D264" s="5" t="inlineStr">
@@ -23288,12 +23288,12 @@
       </c>
       <c r="E264" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Rosemont-La Petite-Patrie, Montréal)</t>
+          <t>6617, Rue Saint-Hubert, app. 201, Montréal</t>
         </is>
       </c>
       <c r="F264" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2175</t>
         </is>
       </c>
       <c r="G264" s="5" t="inlineStr">
@@ -23303,7 +23303,7 @@
       </c>
       <c r="H264" s="5" t="inlineStr">
         <is>
-          <t>3 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I264" s="5" t="inlineStr">
@@ -23313,27 +23313,27 @@
       </c>
       <c r="J264" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K264" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L264" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M264" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N264" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1613584236892605</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/26894928</t>
         </is>
       </c>
       <c r="O264" s="5" t="inlineStr">
@@ -23343,12 +23343,12 @@
       </c>
       <c r="P264" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (« Logement 5 1/2 rénové Rosemont - 3 chambres + bureau »), aucune adresse ni description détaillée disponible via le scraper. Nombre de chambres selon le titre (3 + bureau). Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Entièrement rénové (finitions contemporaines), semi-meublé, climatisation et internet inclus, animaux acceptés sous conditions, disponible 2 jours après acceptation, en plein Plaza St-Hubert, proche marché Jean-Talon et Petite Italie, Walk Score 97. Balcon et superficie non précisés.</t>
         </is>
       </c>
       <c r="Q264" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/789845450_1602489944997832_5213134105176151966_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xzqo9iyYcAkQ7kNvwHRvmWj&amp;_nc_oc=Adp04UM8mMS7TYZztbruBwtONw22BOWfpCFSRMezlhO7JaSrV4L2CIIxMvRmLg4IrzQ&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=iDnTU3IQw0eGZCC-IJSGrw&amp;_nc_ss=7f2a8&amp;oh=00_AQKWwqFPn5wiyRr8UhOqIiE2fW-83zbjH04dhSzspmsjgw&amp;oe=6A9A671F</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4631F1DDDDDDDDDDC&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -23365,7 +23365,7 @@
       </c>
       <c r="C265" s="6" t="inlineStr">
         <is>
-          <t>4½ rénové (2 chambres), semi-meublé - Plaza St-Hubert (Rosemont), près du métro Beaubien</t>
+          <t>4½ (2 chambres) - secteur résidentiel calme, 23e Avenue (Rosemont)</t>
         </is>
       </c>
       <c r="D265" s="5" t="inlineStr">
@@ -23375,12 +23375,12 @@
       </c>
       <c r="E265" s="5" t="inlineStr">
         <is>
-          <t>6617, Rue Saint-Hubert, app. 201, Montréal</t>
+          <t>6001, 23e Avenue, app. 3, Montréal</t>
         </is>
       </c>
       <c r="F265" s="5" t="inlineStr">
         <is>
-          <t>2175</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G265" s="5" t="inlineStr">
@@ -23400,7 +23400,7 @@
       </c>
       <c r="J265" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>Beaubien ou Rosemont (estimé)</t>
         </is>
       </c>
       <c r="K265" s="5" t="inlineStr">
@@ -23410,7 +23410,7 @@
       </c>
       <c r="L265" s="5" t="inlineStr">
         <is>
-          <t>5 (estimé)</t>
+          <t>9 (estimé)</t>
         </is>
       </c>
       <c r="M265" s="5" t="inlineStr">
@@ -23420,7 +23420,7 @@
       </c>
       <c r="N265" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/26894928</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/22497736</t>
         </is>
       </c>
       <c r="O265" s="5" t="inlineStr">
@@ -23430,12 +23430,12 @@
       </c>
       <c r="P265" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové (finitions contemporaines), semi-meublé, climatisation et internet inclus, animaux acceptés sous conditions, disponible 2 jours après acceptation, en plein Plaza St-Hubert, proche marché Jean-Talon et Petite Italie, Walk Score 97. Balcon et superficie non précisés.</t>
+          <t>Bien aménagé, lumineux, finitions soignées, secteur résidentiel paisible près parcs/commerces/écoles, disponible 5 jours après acceptation, Walk Score 85. Balcon, animaux et chauffage non précisés dans l'annonce.</t>
         </is>
       </c>
       <c r="Q265" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4631F1DDDDDDDDDDC&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4AE812DDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -23452,22 +23452,22 @@
       </c>
       <c r="C266" s="6" t="inlineStr">
         <is>
-          <t>4½ (2 chambres) - secteur résidentiel calme, 23e Avenue (Rosemont)</t>
+          <t>4½ (2 chambres) - rue De La Roche (Plateau)</t>
         </is>
       </c>
       <c r="D266" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E266" s="5" t="inlineStr">
         <is>
-          <t>6001, 23e Avenue, app. 3, Montréal</t>
+          <t>4417, Rue De La Roche, app. 4, Montréal</t>
         </is>
       </c>
       <c r="F266" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G266" s="5" t="inlineStr">
@@ -23487,7 +23487,7 @@
       </c>
       <c r="J266" s="5" t="inlineStr">
         <is>
-          <t>Beaubien ou Rosemont (estimé)</t>
+          <t>Mont-Royal (estimé)</t>
         </is>
       </c>
       <c r="K266" s="5" t="inlineStr">
@@ -23497,7 +23497,7 @@
       </c>
       <c r="L266" s="5" t="inlineStr">
         <is>
-          <t>9 (estimé)</t>
+          <t>10 (estimé)</t>
         </is>
       </c>
       <c r="M266" s="5" t="inlineStr">
@@ -23507,7 +23507,7 @@
       </c>
       <c r="N266" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/22497736</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14734354</t>
         </is>
       </c>
       <c r="O266" s="5" t="inlineStr">
@@ -23517,19 +23517,19 @@
       </c>
       <c r="P266" s="6" t="inlineStr">
         <is>
-          <t>Bien aménagé, lumineux, finitions soignées, secteur résidentiel paisible près parcs/commerces/écoles, disponible 5 jours après acceptation, Walk Score 85. Balcon, animaux et chauffage non précisés dans l'annonce.</t>
+          <t>Peu de détails dans l'annonce (balcon, superficie, animaux et chauffage non précisés), disponible 24 août 2026, Walk Score 99, secteur à confirmer avant de contacter.</t>
         </is>
       </c>
       <c r="Q266" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4AE812DDDDDDDDDD2&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA2DDB74DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="267">
       <c r="A267" s="5" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-23</t>
         </is>
       </c>
       <c r="B267" s="5" t="inlineStr">
@@ -23539,7 +23539,7 @@
       </c>
       <c r="C267" s="6" t="inlineStr">
         <is>
-          <t>4½ (2 chambres) - rue De La Roche (Plateau)</t>
+          <t>2 chambres rénové, près de la rue Mont-Royal et du métro Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D267" s="5" t="inlineStr">
@@ -23549,12 +23549,12 @@
       </c>
       <c r="E267" s="5" t="inlineStr">
         <is>
-          <t>4417, Rue De La Roche, app. 4, Montréal</t>
+          <t>4408, Avenue de l'Hôtel-de-Ville, Montréal</t>
         </is>
       </c>
       <c r="F267" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G267" s="5" t="inlineStr">
@@ -23574,7 +23574,7 @@
       </c>
       <c r="J267" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal (estimé)</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K267" s="5" t="inlineStr">
@@ -23584,17 +23584,17 @@
       </c>
       <c r="L267" s="5" t="inlineStr">
         <is>
-          <t>10 (estimé)</t>
+          <t>5 (estimé)</t>
         </is>
       </c>
       <c r="M267" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N267" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14734354</t>
+          <t>https://www.facebook.com/marketplace/item/3643447005808131</t>
         </is>
       </c>
       <c r="O267" s="5" t="inlineStr">
@@ -23604,19 +23604,19 @@
       </c>
       <c r="P267" s="6" t="inlineStr">
         <is>
-          <t>Peu de détails dans l'annonce (balcon, superficie, animaux et chauffage non précisés), disponible 24 août 2026, Walk Score 99, secteur à confirmer avant de contacter.</t>
+          <t>Nouvellement rénové, meublé (table, chaises, canapé, lits), climatisation incluse, isolation phonique/thermique complète, plafonds hauts, animaux acceptés. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q267" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA2DDB74DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/769082955_1572138077922196_3928924517892675151_n.jpg?stp=c0.169.1536.1536a_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=5lbjrhSykR4Q7kNvwGXZEsS&amp;_nc_oc=AdosPHcT82UDB5JXJB3hFRrzA2ywy8Iz4eDC9_v14IG5fPngcGQrop8r6fkrAZcfxOg&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=hnqIHFjbxMu6V7YVFERN2g&amp;_nc_ss=7f2a8&amp;oh=00_AQFUCFiOoITnnQEKag8_p25qfElq9MW43hMXPo8TnhpJ_g&amp;oe=6A91378D</t>
         </is>
       </c>
     </row>
     <row r="268">
       <c r="A268" s="5" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B268" s="5" t="inlineStr">
@@ -23626,22 +23626,22 @@
       </c>
       <c r="C268" s="6" t="inlineStr">
         <is>
-          <t>2 chambres rénové, près de la rue Mont-Royal et du métro Mont-Royal (Marketplace)</t>
+          <t>Appartement 5½ (Hochelaga) - infos limitées, à vérifier via Facebook Marketplace</t>
         </is>
       </c>
       <c r="D268" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E268" s="5" t="inlineStr">
         <is>
-          <t>4408, Avenue de l'Hôtel-de-Ville, Montréal</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F268" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>1995</t>
         </is>
       </c>
       <c r="G268" s="5" t="inlineStr">
@@ -23651,7 +23651,7 @@
       </c>
       <c r="H268" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I268" s="5" t="inlineStr">
@@ -23661,17 +23661,17 @@
       </c>
       <c r="J268" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>n/d (secteur Hochelaga)</t>
         </is>
       </c>
       <c r="K268" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L268" s="5" t="inlineStr">
         <is>
-          <t>5 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M268" s="5" t="inlineStr">
@@ -23681,7 +23681,7 @@
       </c>
       <c r="N268" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/3643447005808131</t>
+          <t>https://www.facebook.com/marketplace/item/1020807880801669</t>
         </is>
       </c>
       <c r="O268" s="5" t="inlineStr">
@@ -23691,19 +23691,19 @@
       </c>
       <c r="P268" s="6" t="inlineStr">
         <is>
-          <t>Nouvellement rénové, meublé (table, chaises, canapé, lits), climatisation incluse, isolation phonique/thermique complète, plafonds hauts, animaux acceptés. Lien Facebook (connexion requise)</t>
+          <t>Fiche Marketplace très peu détaillée (titre et prix seulement, pas de description ni superficie). Chambres estimées à 3 d'après le type 5½. Le lien exige une connexion Facebook pour voir les détails complets.</t>
         </is>
       </c>
       <c r="Q268" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/769082955_1572138077922196_3928924517892675151_n.jpg?stp=c0.169.1536.1536a_dst-jpg_tt6&amp;cstp=mx1536x1536&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=5lbjrhSykR4Q7kNvwGXZEsS&amp;_nc_oc=AdosPHcT82UDB5JXJB3hFRrzA2ywy8Iz4eDC9_v14IG5fPngcGQrop8r6fkrAZcfxOg&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=hnqIHFjbxMu6V7YVFERN2g&amp;_nc_ss=7f2a8&amp;oh=00_AQFUCFiOoITnnQEKag8_p25qfElq9MW43hMXPo8TnhpJ_g&amp;oe=6A91378D</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/740733947_28734879242768603_2405899251014488449_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q9ViAyeDpUAQ7kNvwFF85BL&amp;_nc_oc=Adr4Bry90yP1945bAQ7iQ52U9LuxXUfcltCcAJNNZMjNUaTJQ7tsFLsd_jtuJfl42Ps&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=rTvNKBKykO1Kn418ORNEfA&amp;_nc_ss=7f2a8&amp;oh=00_AQHwScRvAsPs8uZWD-UEV1uK_8325MQziNdaYa1h63-U7A&amp;oe=6A8FDC27</t>
         </is>
       </c>
     </row>
     <row r="269">
       <c r="A269" s="5" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B269" s="5" t="inlineStr">
@@ -23713,22 +23713,22 @@
       </c>
       <c r="C269" s="6" t="inlineStr">
         <is>
-          <t>Appartement 5½ (Hochelaga) - infos limitées, à vérifier via Facebook Marketplace</t>
+          <t>Appartement 2 chambres + bureau, quartier central Plateau, à ~11 min du métro Sherbrooke (Marketplace)</t>
         </is>
       </c>
       <c r="D269" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E269" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>3984 Rue de Bullion, Montréal, QC H2W 2E4</t>
         </is>
       </c>
       <c r="F269" s="5" t="inlineStr">
         <is>
-          <t>1995</t>
+          <t>2300</t>
         </is>
       </c>
       <c r="G269" s="5" t="inlineStr">
@@ -23738,59 +23738,59 @@
       </c>
       <c r="H269" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I269" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J269" s="5" t="inlineStr">
+        <is>
+          <t>Sherbrooke</t>
+        </is>
+      </c>
+      <c r="K269" s="5" t="inlineStr">
+        <is>
+          <t>orange</t>
+        </is>
+      </c>
+      <c r="L269" s="5" t="inlineStr">
+        <is>
+          <t>11</t>
+        </is>
+      </c>
+      <c r="M269" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="N269" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/1528694045314689</t>
+        </is>
+      </c>
+      <c r="O269" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I269" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J269" s="5" t="inlineStr">
-        <is>
-          <t>n/d (secteur Hochelaga)</t>
-        </is>
-      </c>
-      <c r="K269" s="5" t="inlineStr">
-        <is>
-          <t>verte</t>
-        </is>
-      </c>
-      <c r="L269" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M269" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N269" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1020807880801669</t>
-        </is>
-      </c>
-      <c r="O269" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="P269" s="6" t="inlineStr">
         <is>
-          <t>Fiche Marketplace très peu détaillée (titre et prix seulement, pas de description ni superficie). Chambres estimées à 3 d'après le type 5½. Le lien exige une connexion Facebook pour voir les détails complets.</t>
+          <t>Deux chambres fermees + un espace de bureau, electromenagers inclus, bail 1 an, disponible maintenant, quartier central (Walk Score 100, Bike Score 98). Superficie non indiquee. Lien Facebook (connexion requise).</t>
         </is>
       </c>
       <c r="Q269" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/740733947_28734879242768603_2405899251014488449_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=105&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q9ViAyeDpUAQ7kNvwFF85BL&amp;_nc_oc=Adr4Bry90yP1945bAQ7iQ52U9LuxXUfcltCcAJNNZMjNUaTJQ7tsFLsd_jtuJfl42Ps&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=rTvNKBKykO1Kn418ORNEfA&amp;_nc_ss=7f2a8&amp;oh=00_AQHwScRvAsPs8uZWD-UEV1uK_8325MQziNdaYa1h63-U7A&amp;oe=6A8FDC27</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/722994642_10164255701674834_4384640404152492239_n.jpg?stp=c342.0.1365.1365a_dst-jpg_tt6&amp;cstp=mx1365x1365&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=P20jq1k6qjIQ7kNvwF35WB_&amp;_nc_oc=AdrWOhKe-TO43O_pi7-zm4f94i1vfAPIWDFFxE3h49ZzbSfBqp_EeJowVqfsNEyEzmY&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=-RRMTc1fIutY57-pjw9YmQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHvo5JUjbFeFE0mNam3RiJtgV0tjwf8rAM1aebC8RWpDQ&amp;oe=6A8E14C9</t>
         </is>
       </c>
     </row>
     <row r="270">
       <c r="A270" s="5" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B270" s="5" t="inlineStr">
@@ -23800,22 +23800,22 @@
       </c>
       <c r="C270" s="6" t="inlineStr">
         <is>
-          <t>Appartement 2 chambres + bureau, quartier central Plateau, à ~11 min du métro Sherbrooke (Marketplace)</t>
+          <t>5½ rénové (2 chambres), garde-robes walk-in - secteur Villeray, à 5 min du métro Jarry</t>
         </is>
       </c>
       <c r="D270" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E270" s="5" t="inlineStr">
         <is>
-          <t>3984 Rue de Bullion, Montréal, QC H2W 2E4</t>
+          <t>n/d (Montréal, QC H2R 2P3)</t>
         </is>
       </c>
       <c r="F270" s="5" t="inlineStr">
         <is>
-          <t>2300</t>
+          <t>1900</t>
         </is>
       </c>
       <c r="G270" s="5" t="inlineStr">
@@ -23830,12 +23830,12 @@
       </c>
       <c r="I270" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J270" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Jarry</t>
         </is>
       </c>
       <c r="K270" s="5" t="inlineStr">
@@ -23845,7 +23845,7 @@
       </c>
       <c r="L270" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M270" s="5" t="inlineStr">
@@ -23855,7 +23855,7 @@
       </c>
       <c r="N270" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1528694045314689</t>
+          <t>https://www.facebook.com/marketplace/item/1318066247058264</t>
         </is>
       </c>
       <c r="O270" s="5" t="inlineStr">
@@ -23865,19 +23865,19 @@
       </c>
       <c r="P270" s="6" t="inlineStr">
         <is>
-          <t>Deux chambres fermees + un espace de bureau, electromenagers inclus, bail 1 an, disponible maintenant, quartier central (Walk Score 100, Bike Score 98). Superficie non indiquee. Lien Facebook (connexion requise).</t>
+          <t>Entièrement rénové (cuisine avec îlot, planchers refaits), chambre principale avec walk-in, 2e chambre avec grand garde-robe, thermopompe, porte-patio vers cour arrière (pas de balcon), à distance de marche du métro Jarry et du marché Jean-Talon, références demandées, aucun animal, disponible 1er oct. 2026, bail 1 an. Lien Facebook (connexion requise).</t>
         </is>
       </c>
       <c r="Q270" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/722994642_10164255701674834_4384640404152492239_n.jpg?stp=c342.0.1365.1365a_dst-jpg_tt6&amp;cstp=mx1365x1365&amp;ctp=s565x565&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=P20jq1k6qjIQ7kNvwF35WB_&amp;_nc_oc=AdrWOhKe-TO43O_pi7-zm4f94i1vfAPIWDFFxE3h49ZzbSfBqp_EeJowVqfsNEyEzmY&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=-RRMTc1fIutY57-pjw9YmQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHvo5JUjbFeFE0mNam3RiJtgV0tjwf8rAM1aebC8RWpDQ&amp;oe=6A8E14C9</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/730304009_10243338752987620_3251931066748678009_n.jpg?stp=c341.0.1367.1367a_dst-jpg_tt6&amp;cstp=mx1367x1367&amp;ctp=s565x565&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=T1M2AeYt3WkQ7kNvwEbtDR9&amp;_nc_oc=AdqdPqtbLbupPJRjBJ9G6l5MxrQhR9IhCxSGNw-xvzoSzkXhl2b7yw4yEMa1hIVXQLo&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=gi1y626B7giI3AkvJxbp7A&amp;_nc_ss=7f2a8&amp;oh=00_AQHDh36TzcRlsSalStNzCi2WPYfPNl7gzA_gMGdg3e-VhQ&amp;oe=6A8B7951</t>
         </is>
       </c>
     </row>
     <row r="271">
       <c r="A271" s="5" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B271" s="5" t="inlineStr">
@@ -23887,22 +23887,22 @@
       </c>
       <c r="C271" s="6" t="inlineStr">
         <is>
-          <t>5½ rénové (2 chambres), garde-robes walk-in - secteur Villeray, à 5 min du métro Jarry</t>
+          <t>5 1/2 (2 chambres) avec bureau, 2e étage - rue Saint-Viateur Ouest (Mile-End/Plateau)</t>
         </is>
       </c>
       <c r="D271" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E271" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2R 2P3)</t>
+          <t>229, Rue Saint-Viateur Ouest, app. 3, Montréal</t>
         </is>
       </c>
       <c r="F271" s="5" t="inlineStr">
         <is>
-          <t>1900</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G271" s="5" t="inlineStr">
@@ -23917,12 +23917,12 @@
       </c>
       <c r="I271" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J271" s="5" t="inlineStr">
         <is>
-          <t>Jarry</t>
+          <t>Rosemont (estimé)</t>
         </is>
       </c>
       <c r="K271" s="5" t="inlineStr">
@@ -23932,17 +23932,17 @@
       </c>
       <c r="L271" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>12 (estimé)</t>
         </is>
       </c>
       <c r="M271" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N271" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1318066247058264</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/12176453</t>
         </is>
       </c>
       <c r="O271" s="5" t="inlineStr">
@@ -23952,19 +23952,19 @@
       </c>
       <c r="P271" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové (cuisine avec îlot, planchers refaits), chambre principale avec walk-in, 2e chambre avec grand garde-robe, thermopompe, porte-patio vers cour arrière (pas de balcon), à distance de marche du métro Jarry et du marché Jean-Talon, références demandées, aucun animal, disponible 1er oct. 2026, bail 1 an. Lien Facebook (connexion requise).</t>
+          <t>Salle a manger, bureau, semi-meuble (frigo et cuisiniere inclus), locataire paie chauffage et electricite, animaux et fumeurs non acceptes, disponible 5 jours apres acceptation, secteur Mile-End/Plateau, Walk Score 100</t>
         </is>
       </c>
       <c r="Q271" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.30808-6/730304009_10243338752987620_3251931066748678009_n.jpg?stp=c341.0.1367.1367a_dst-jpg_tt6&amp;cstp=mx1367x1367&amp;ctp=s565x565&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=454cf4&amp;_nc_ohc=T1M2AeYt3WkQ7kNvwEbtDR9&amp;_nc_oc=AdqdPqtbLbupPJRjBJ9G6l5MxrQhR9IhCxSGNw-xvzoSzkXhl2b7yw4yEMa1hIVXQLo&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=gi1y626B7giI3AkvJxbp7A&amp;_nc_ss=7f2a8&amp;oh=00_AQHDh36TzcRlsSalStNzCi2WPYfPNl7gzA_gMGdg3e-VhQ&amp;oe=6A8B7951</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4189D5DDDDDDDDDDB&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="272">
       <c r="A272" s="5" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B272" s="5" t="inlineStr">
@@ -23974,22 +23974,22 @@
       </c>
       <c r="C272" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 (2 chambres) avec bureau, 2e étage - rue Saint-Viateur Ouest (Mile-End/Plateau)</t>
+          <t>Logement 6 1/2 à louer dans Villeray (Marketplace)</t>
         </is>
       </c>
       <c r="D272" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E272" s="5" t="inlineStr">
         <is>
-          <t>229, Rue Saint-Viateur Ouest, app. 3, Montréal</t>
+          <t>n/d (secteur Villeray, Montréal)</t>
         </is>
       </c>
       <c r="F272" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G272" s="5" t="inlineStr">
@@ -23999,7 +23999,7 @@
       </c>
       <c r="H272" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3 (estimé)</t>
         </is>
       </c>
       <c r="I272" s="5" t="inlineStr">
@@ -24009,27 +24009,27 @@
       </c>
       <c r="J272" s="5" t="inlineStr">
         <is>
-          <t>Rosemont (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K272" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L272" s="5" t="inlineStr">
         <is>
-          <t>12 (estimé)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M272" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N272" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/12176453</t>
+          <t>https://www.facebook.com/marketplace/item/1020450404083699</t>
         </is>
       </c>
       <c r="O272" s="5" t="inlineStr">
@@ -24039,19 +24039,19 @@
       </c>
       <c r="P272" s="6" t="inlineStr">
         <is>
-          <t>Salle a manger, bureau, semi-meuble (frigo et cuisiniere inclus), locataire paie chauffage et electricite, animaux et fumeurs non acceptes, disponible 5 jours apres acceptation, secteur Mile-End/Plateau, Walk Score 100</t>
+          <t>Annonce titre seulement (« Logement a loué 6 1/2 dans villeray »), aucune description ni adresse disponible via le scraper. Nombre de chambres estimé à 3 selon la nomenclature standard d'un 6½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q272" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA4189D5DDDDDDDDDDB&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/763805631_1503784241770162_4967544372375745805_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=101&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=jGqmb0NgpJoQ7kNvwFH3YjO&amp;_nc_oc=AdoY1EsSNcq7zLnPmamdgZYnFxscFtqiBT5k0ZKtBAzp-lkY2KX7KLoaQ55MsEJFKcc&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=Jh4pE02jeamMrq9aD_orfQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHVB3CnZ5QJ3Jhj2o-a6Li1sE8vgz3c5ABW_l7p_nT4sA&amp;oe=6A790FD8</t>
         </is>
       </c>
     </row>
     <row r="273">
       <c r="A273" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-23</t>
         </is>
       </c>
       <c r="B273" s="5" t="inlineStr">
@@ -24061,22 +24061,22 @@
       </c>
       <c r="C273" s="6" t="inlineStr">
         <is>
-          <t>Logement 6 1/2 à louer dans Villeray (Marketplace)</t>
+          <t>2 chambres - rue De Lanaudière (Rosemont), à 6 min du métro Jean-Talon</t>
         </is>
       </c>
       <c r="D273" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E273" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Villeray, Montréal)</t>
+          <t>6583, Rue De Lanaudière, Montréal</t>
         </is>
       </c>
       <c r="F273" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1945</t>
         </is>
       </c>
       <c r="G273" s="5" t="inlineStr">
@@ -24086,7 +24086,7 @@
       </c>
       <c r="H273" s="5" t="inlineStr">
         <is>
-          <t>3 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I273" s="5" t="inlineStr">
@@ -24096,27 +24096,27 @@
       </c>
       <c r="J273" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Jean-Talon</t>
         </is>
       </c>
       <c r="K273" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>orange/bleue</t>
         </is>
       </c>
       <c r="L273" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>6</t>
         </is>
       </c>
       <c r="M273" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N273" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1020450404083699</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20257676</t>
         </is>
       </c>
       <c r="O273" s="5" t="inlineStr">
@@ -24126,12 +24126,12 @@
       </c>
       <c r="P273" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (« Logement a loué 6 1/2 dans villeray »), aucune description ni adresse disponible via le scraper. Nombre de chambres estimé à 3 selon la nomenclature standard d'un 6½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Chauffage central inclus + 5 électroménagers, quintuplex de 1932, disponible 1er sept. 2026, Walk Score 94</t>
         </is>
       </c>
       <c r="Q273" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/763805631_1503784241770162_4967544372375745805_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=101&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=jGqmb0NgpJoQ7kNvwFH3YjO&amp;_nc_oc=AdoY1EsSNcq7zLnPmamdgZYnFxscFtqiBT5k0ZKtBAzp-lkY2KX7KLoaQ55MsEJFKcc&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=Jh4pE02jeamMrq9aD_orfQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHVB3CnZ5QJ3Jhj2o-a6Li1sE8vgz3c5ABW_l7p_nT4sA&amp;oe=6A790FD8</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15EA61DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -24148,22 +24148,22 @@
       </c>
       <c r="C274" s="6" t="inlineStr">
         <is>
-          <t>2 chambres - rue De Lanaudière (Rosemont), à 6 min du métro Jean-Talon</t>
+          <t>2 chambres avec cour privée - rue Demers (Plateau), près du métro Laurier</t>
         </is>
       </c>
       <c r="D274" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E274" s="5" t="inlineStr">
         <is>
-          <t>6583, Rue De Lanaudière, Montréal</t>
+          <t>170, Rue Demers, Montréal</t>
         </is>
       </c>
       <c r="F274" s="5" t="inlineStr">
         <is>
-          <t>1945</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G274" s="5" t="inlineStr">
@@ -24178,22 +24178,22 @@
       </c>
       <c r="I274" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J274" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon</t>
+          <t>Laurier</t>
         </is>
       </c>
       <c r="K274" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L274" s="5" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>8-10 (estimé)</t>
         </is>
       </c>
       <c r="M274" s="5" t="inlineStr">
@@ -24203,7 +24203,7 @@
       </c>
       <c r="N274" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/20257676</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/15892581</t>
         </is>
       </c>
       <c r="O274" s="5" t="inlineStr">
@@ -24213,19 +24213,19 @@
       </c>
       <c r="P274" s="6" t="inlineStr">
         <is>
-          <t>Chauffage central inclus + 5 électroménagers, quintuplex de 1932, disponible 1er sept. 2026, Walk Score 94</t>
+          <t>Thermopompe murale incluse, meublé, cour privée (pas de balcon), animaux non acceptés, secteur Mile End, Walk Score 99</t>
         </is>
       </c>
       <c r="Q274" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA15EA61DDDDDDDDDDE&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADFCE64DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="275">
       <c r="A275" s="5" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B275" s="5" t="inlineStr">
@@ -24235,7 +24235,7 @@
       </c>
       <c r="C275" s="6" t="inlineStr">
         <is>
-          <t>2 chambres avec cour privée - rue Demers (Plateau), près du métro Laurier</t>
+          <t>Spacieux 4½ rénové, 2 chambres - avenue Henri-Julien (Plateau), à 2 min du métro Laurier</t>
         </is>
       </c>
       <c r="D275" s="5" t="inlineStr">
@@ -24245,12 +24245,12 @@
       </c>
       <c r="E275" s="5" t="inlineStr">
         <is>
-          <t>170, Rue Demers, Montréal</t>
+          <t>5010, Avenue Henri-Julien, Montréal</t>
         </is>
       </c>
       <c r="F275" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G275" s="5" t="inlineStr">
@@ -24265,7 +24265,7 @@
       </c>
       <c r="I275" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J275" s="5" t="inlineStr">
@@ -24280,7 +24280,7 @@
       </c>
       <c r="L275" s="5" t="inlineStr">
         <is>
-          <t>8-10 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="M275" s="5" t="inlineStr">
@@ -24290,7 +24290,7 @@
       </c>
       <c r="N275" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/15892581</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/13104221</t>
         </is>
       </c>
       <c r="O275" s="5" t="inlineStr">
@@ -24300,12 +24300,12 @@
       </c>
       <c r="P275" s="6" t="inlineStr">
         <is>
-          <t>Thermopompe murale incluse, meublé, cour privée (pas de balcon), animaux non acceptés, secteur Mile End, Walk Score 99</t>
+          <t>Cuisine et salle de bain rénovées, hauts plafonds, immeuble de 1910, chats acceptés, disponible 7 jours après acceptation, Walk Score 99</t>
         </is>
       </c>
       <c r="Q275" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADFCE64DDDDDDDDDD1&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA41C20BDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -24322,7 +24322,7 @@
       </c>
       <c r="C276" s="6" t="inlineStr">
         <is>
-          <t>Spacieux 4½ rénové, 2 chambres - avenue Henri-Julien (Plateau), à 2 min du métro Laurier</t>
+          <t>4½ avec cour arrière privée - rue Rivard (Plateau), à quelques pas du métro Mont-Royal</t>
         </is>
       </c>
       <c r="D276" s="5" t="inlineStr">
@@ -24332,7 +24332,7 @@
       </c>
       <c r="E276" s="5" t="inlineStr">
         <is>
-          <t>5010, Avenue Henri-Julien, Montréal</t>
+          <t>4452, Rue Rivard, Montréal</t>
         </is>
       </c>
       <c r="F276" s="5" t="inlineStr">
@@ -24352,12 +24352,12 @@
       </c>
       <c r="I276" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>non</t>
         </is>
       </c>
       <c r="J276" s="5" t="inlineStr">
         <is>
-          <t>Laurier</t>
+          <t>Mont-Royal</t>
         </is>
       </c>
       <c r="K276" s="5" t="inlineStr">
@@ -24367,7 +24367,7 @@
       </c>
       <c r="L276" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3 (estimé)</t>
         </is>
       </c>
       <c r="M276" s="5" t="inlineStr">
@@ -24377,7 +24377,7 @@
       </c>
       <c r="N276" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/13104221</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14560801</t>
         </is>
       </c>
       <c r="O276" s="5" t="inlineStr">
@@ -24387,19 +24387,19 @@
       </c>
       <c r="P276" s="6" t="inlineStr">
         <is>
-          <t>Cuisine et salle de bain rénovées, hauts plafonds, immeuble de 1910, chats acceptés, disponible 7 jours après acceptation, Walk Score 99</t>
+          <t>Cour arrière privée, lumineux et bien entretenu, Walk Score 100, animaux acceptés sous conditions, disponible 1er août 2026</t>
         </is>
       </c>
       <c r="Q276" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA41C20BDDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA44883FDDDDDDDDDDA&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="277">
       <c r="A277" s="5" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B277" s="5" t="inlineStr">
@@ -24409,22 +24409,22 @@
       </c>
       <c r="C277" s="6" t="inlineStr">
         <is>
-          <t>4½ avec cour arrière privée - rue Rivard (Plateau), à quelques pas du métro Mont-Royal</t>
+          <t>Grand 6 1/2, 2 chambres - rue Jean-Talon Est (Rosemont, près marché Jean-Talon)</t>
         </is>
       </c>
       <c r="D277" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E277" s="5" t="inlineStr">
         <is>
-          <t>4452, Rue Rivard, Montréal</t>
+          <t>274, Rue Jean-Talon Est, app. 302, Montréal</t>
         </is>
       </c>
       <c r="F277" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G277" s="5" t="inlineStr">
@@ -24439,22 +24439,22 @@
       </c>
       <c r="I277" s="5" t="inlineStr">
         <is>
-          <t>non</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="J277" s="5" t="inlineStr">
         <is>
-          <t>Mont-Royal</t>
+          <t>Jean-Talon</t>
         </is>
       </c>
       <c r="K277" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>orange/bleue</t>
         </is>
       </c>
       <c r="L277" s="5" t="inlineStr">
         <is>
-          <t>3 (estimé)</t>
+          <t>11</t>
         </is>
       </c>
       <c r="M277" s="5" t="inlineStr">
@@ -24464,7 +24464,7 @@
       </c>
       <c r="N277" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/14560801</t>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/14545078</t>
         </is>
       </c>
       <c r="O277" s="5" t="inlineStr">
@@ -24474,19 +24474,19 @@
       </c>
       <c r="P277" s="6" t="inlineStr">
         <is>
-          <t>Cour arrière privée, lumineux et bien entretenu, Walk Score 100, animaux acceptés sous conditions, disponible 1er août 2026</t>
+          <t>6 pièces au total, concept ouvert, comptoirs de quartz, walk score 100, dispo 1er juillet 2026, près du marché Jean-Talon, superficie non précisée</t>
         </is>
       </c>
       <c r="Q277" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DA44883FDDDDDDDDDDA&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADE4013DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="278">
       <c r="A278" s="5" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B278" s="5" t="inlineStr">
@@ -24496,7 +24496,7 @@
       </c>
       <c r="C278" s="6" t="inlineStr">
         <is>
-          <t>Grand 6 1/2, 2 chambres - rue Jean-Talon Est (Rosemont, près marché Jean-Talon)</t>
+          <t>Cession de bail 7½, Rosemont-La Petite-Patrie (Marketplace)</t>
         </is>
       </c>
       <c r="D278" s="5" t="inlineStr">
@@ -24506,12 +24506,12 @@
       </c>
       <c r="E278" s="5" t="inlineStr">
         <is>
-          <t>274, Rue Jean-Talon Est, app. 302, Montréal</t>
+          <t>n/d (Montréal, QC H2G 1T5)</t>
         </is>
       </c>
       <c r="F278" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2060</t>
         </is>
       </c>
       <c r="G278" s="5" t="inlineStr">
@@ -24521,7 +24521,7 @@
       </c>
       <c r="H278" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I278" s="5" t="inlineStr">
@@ -24531,27 +24531,27 @@
       </c>
       <c r="J278" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K278" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L278" s="5" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M278" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N278" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/14545078</t>
+          <t>https://www.facebook.com/marketplace/item/1375157431101110</t>
         </is>
       </c>
       <c r="O278" s="5" t="inlineStr">
@@ -24561,12 +24561,12 @@
       </c>
       <c r="P278" s="6" t="inlineStr">
         <is>
-          <t>6 pièces au total, concept ouvert, comptoirs de quartz, walk score 100, dispo 1er juillet 2026, près du marché Jean-Talon, superficie non précisée</t>
+          <t>Cession de bail. Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q278" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADE4013DDDDDDDDDDC&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/702670571_1710902896599779_1133264177050399379_n.jpg?stp=c0.86.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=akFqSvK3rfAQ7kNvwG-Cqey&amp;_nc_oc=Adrp5N9Rg13Pf-obfNZqB1ZqwyOcgjJji8vk0ggvRJiA9uCo-xDJXuQAit6O7YIGPW0&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQBG56r36JKH2gkm4Baddcm0ylaFria-4p9Il0vYABnyMg&amp;oe=6A607060</t>
         </is>
       </c>
     </row>
@@ -24583,22 +24583,22 @@
       </c>
       <c r="C279" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail 7½, Rosemont-La Petite-Patrie (Marketplace)</t>
+          <t>Condo 2 chambres semi-meublé, stationnement intérieur - rue Villeray, à 9 min du métro Fabre</t>
         </is>
       </c>
       <c r="D279" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Villeray</t>
         </is>
       </c>
       <c r="E279" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC H2G 1T5)</t>
+          <t>1414 Rue Villeray, app. 105, Montréal</t>
         </is>
       </c>
       <c r="F279" s="5" t="inlineStr">
         <is>
-          <t>2060</t>
+          <t>2350</t>
         </is>
       </c>
       <c r="G279" s="5" t="inlineStr">
@@ -24608,59 +24608,59 @@
       </c>
       <c r="H279" s="5" t="inlineStr">
         <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="I279" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J279" s="5" t="inlineStr">
+        <is>
+          <t>Fabre</t>
+        </is>
+      </c>
+      <c r="K279" s="5" t="inlineStr">
+        <is>
+          <t>bleue</t>
+        </is>
+      </c>
+      <c r="L279" s="5" t="inlineStr">
+        <is>
+          <t>9</t>
+        </is>
+      </c>
+      <c r="M279" s="5" t="inlineStr">
+        <is>
+          <t>Centris</t>
+        </is>
+      </c>
+      <c r="N279" s="7" t="inlineStr">
+        <is>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-villeray-saint-michel-parc-extension/25583093</t>
+        </is>
+      </c>
+      <c r="O279" s="5" t="inlineStr">
+        <is>
           <t>3</t>
         </is>
       </c>
-      <c r="I279" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J279" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K279" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L279" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M279" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N279" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1375157431101110</t>
-        </is>
-      </c>
-      <c r="O279" s="5" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
       <c r="P279" s="6" t="inlineStr">
         <is>
-          <t>Cession de bail. Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
+          <t>Immeuble de 2011 (30 unités), RDC, plancher chauffant salle de bain, stationnement intérieur avec borne de recharge, casier de rangement, buanderie commune, terrasse sur le toit, Walk Score 94, dispo 1er juillet 2026</t>
         </is>
       </c>
       <c r="Q279" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/702670571_1710902896599779_1133264177050399379_n.jpg?stp=c0.86.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=akFqSvK3rfAQ7kNvwG-Cqey&amp;_nc_oc=Adrp5N9Rg13Pf-obfNZqB1ZqwyOcgjJji8vk0ggvRJiA9uCo-xDJXuQAit6O7YIGPW0&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQBG56r36JKH2gkm4Baddcm0ylaFria-4p9Il0vYABnyMg&amp;oe=6A607060</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD77D67DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="280">
       <c r="A280" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B280" s="5" t="inlineStr">
@@ -24670,22 +24670,22 @@
       </c>
       <c r="C280" s="6" t="inlineStr">
         <is>
-          <t>Condo 2 chambres semi-meublé, stationnement intérieur - rue Villeray, à 9 min du métro Fabre</t>
+          <t>4½ rénové, 2 chambres, à 3-4 min du métro Sherbrooke</t>
         </is>
       </c>
       <c r="D280" s="5" t="inlineStr">
         <is>
-          <t>Villeray</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E280" s="5" t="inlineStr">
         <is>
-          <t>1414 Rue Villeray, app. 105, Montréal</t>
+          <t>3711 Rue Saint-Urbain, app. A, Montréal</t>
         </is>
       </c>
       <c r="F280" s="5" t="inlineStr">
         <is>
-          <t>2350</t>
+          <t>2292</t>
         </is>
       </c>
       <c r="G280" s="5" t="inlineStr">
@@ -24705,17 +24705,17 @@
       </c>
       <c r="J280" s="5" t="inlineStr">
         <is>
-          <t>Fabre</t>
+          <t>Sherbrooke</t>
         </is>
       </c>
       <c r="K280" s="5" t="inlineStr">
         <is>
-          <t>bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L280" s="5" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>4</t>
         </is>
       </c>
       <c r="M280" s="5" t="inlineStr">
@@ -24725,7 +24725,7 @@
       </c>
       <c r="N280" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-villeray-saint-michel-parc-extension/25583093</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/9588101</t>
         </is>
       </c>
       <c r="O280" s="5" t="inlineStr">
@@ -24735,12 +24735,12 @@
       </c>
       <c r="P280" s="6" t="inlineStr">
         <is>
-          <t>Immeuble de 2011 (30 unités), RDC, plancher chauffant salle de bain, stationnement intérieur avec borne de recharge, casier de rangement, buanderie commune, terrasse sur le toit, Walk Score 94, dispo 1er juillet 2026</t>
+          <t>Cuisine et salle de bain rénovées, plafonds hauts, tous électros inclus, Walk Score 100, dispo 5 jours après acceptation, à 5 min de McGill</t>
         </is>
       </c>
       <c r="Q280" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DAD77D67DDDDDDDDDDB&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6F28A2DDDDDDDDDDB&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
         </is>
       </c>
     </row>
@@ -24757,22 +24757,22 @@
       </c>
       <c r="C281" s="6" t="inlineStr">
         <is>
-          <t>4½ rénové, 2 chambres, à 3-4 min du métro Sherbrooke</t>
+          <t>Appartement meublé haut de gamme - avenue Henri-Julien (Rosemont), près marché Jean-Talon</t>
         </is>
       </c>
       <c r="D281" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E281" s="5" t="inlineStr">
         <is>
-          <t>3711 Rue Saint-Urbain, app. A, Montréal</t>
+          <t>6391 Avenue Henri-Julien, Montréal</t>
         </is>
       </c>
       <c r="F281" s="5" t="inlineStr">
         <is>
-          <t>2292</t>
+          <t>2250</t>
         </is>
       </c>
       <c r="G281" s="5" t="inlineStr">
@@ -24792,17 +24792,17 @@
       </c>
       <c r="J281" s="5" t="inlineStr">
         <is>
-          <t>Sherbrooke</t>
+          <t>Jean-Talon (à vérifier)</t>
         </is>
       </c>
       <c r="K281" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>orange/bleue</t>
         </is>
       </c>
       <c r="L281" s="5" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8 (estimé)</t>
         </is>
       </c>
       <c r="M281" s="5" t="inlineStr">
@@ -24812,7 +24812,7 @@
       </c>
       <c r="N281" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-le-plateau-mont-royal/9588101</t>
+          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/10049540</t>
         </is>
       </c>
       <c r="O281" s="5" t="inlineStr">
@@ -24822,19 +24822,19 @@
       </c>
       <c r="P281" s="6" t="inlineStr">
         <is>
-          <t>Cuisine et salle de bain rénovées, plafonds hauts, tous électros inclus, Walk Score 100, dispo 5 jours après acceptation, à 5 min de McGill</t>
+          <t>Meublé, finitions haut de gamme, pas d'animaux, Walk Score 98, proche marché Jean-Talon et cafés/restos, dispo 1er juin 2026, distance au métro estimée</t>
         </is>
       </c>
       <c r="Q281" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE6F28A2DDDDDDDDDDB&amp;t=pi&amp;w=1024&amp;h=640&amp;sm=c</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADB62FFDDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="282">
       <c r="A282" s="5" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B282" s="5" t="inlineStr">
@@ -24844,22 +24844,22 @@
       </c>
       <c r="C282" s="6" t="inlineStr">
         <is>
-          <t>Appartement meublé haut de gamme - avenue Henri-Julien (Rosemont), près marché Jean-Talon</t>
+          <t>Superbe 2 chambres rénové, rue Beaubien - Petite-Italie</t>
         </is>
       </c>
       <c r="D282" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>La Petite-Patrie</t>
         </is>
       </c>
       <c r="E282" s="5" t="inlineStr">
         <is>
-          <t>6391 Avenue Henri-Julien, Montréal</t>
+          <t>Rue Beaubien (Montréal, QC)</t>
         </is>
       </c>
       <c r="F282" s="5" t="inlineStr">
         <is>
-          <t>2250</t>
+          <t>2050</t>
         </is>
       </c>
       <c r="G282" s="5" t="inlineStr">
@@ -24879,27 +24879,27 @@
       </c>
       <c r="J282" s="5" t="inlineStr">
         <is>
-          <t>Jean-Talon (à vérifier)</t>
+          <t>Beaubien</t>
         </is>
       </c>
       <c r="K282" s="5" t="inlineStr">
         <is>
-          <t>orange/bleue</t>
+          <t>orange</t>
         </is>
       </c>
       <c r="L282" s="5" t="inlineStr">
         <is>
-          <t>8 (estimé)</t>
+          <t>5</t>
         </is>
       </c>
       <c r="M282" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N282" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/fr/condo-appartement~a-louer~montreal-rosemont-la-petite-patrie/10049540</t>
+          <t>https://www.facebook.com/marketplace/item/2219881575422253</t>
         </is>
       </c>
       <c r="O282" s="5" t="inlineStr">
@@ -24909,19 +24909,19 @@
       </c>
       <c r="P282" s="6" t="inlineStr">
         <is>
-          <t>Meublé, finitions haut de gamme, pas d'animaux, Walk Score 98, proche marché Jean-Talon et cafés/restos, dispo 1er juin 2026, distance au métro estimée</t>
+          <t>Entièrement rénové, cour arrière privée, Walk Score 99, à quelques pas de cafés/restos/boulangeries/épiceries fines de la Petite-Italie, à environ 10 min du marché Jean-Talon. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q282" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DADB62FFDDDDDDDDDDD&amp;t=pi&amp;w=640&amp;h=480&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/714823210_969706739294886_222709070726311984_n.jpg?stp=c134.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=111&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q4rmFfALvM0Q7kNvwH2W42u&amp;_nc_oc=AdpINKj09PPc8Re8DxGgY3chRB5RnttQl9NAS-AFL9O8KTqqt1dR9NYx_1WNt0O8lww&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=JqfxygLQ7LNnSdbCmwTgsw&amp;_nc_ss=7f2a8&amp;oh=00_AQDsARrJ7YHo6O-8Zg1v5X3ykFLojfdUxVqQy1Z7t2iyQg&amp;oe=6A5DC11E</t>
         </is>
       </c>
     </row>
     <row r="283">
       <c r="A283" s="5" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B283" s="5" t="inlineStr">
@@ -24931,22 +24931,22 @@
       </c>
       <c r="C283" s="6" t="inlineStr">
         <is>
-          <t>Superbe 2 chambres rénové, rue Beaubien - Petite-Italie</t>
+          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
         </is>
       </c>
       <c r="D283" s="5" t="inlineStr">
         <is>
-          <t>La Petite-Patrie</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E283" s="5" t="inlineStr">
         <is>
-          <t>Rue Beaubien (Montréal, QC)</t>
+          <t>1889 Rue des Carrières, Montréal</t>
         </is>
       </c>
       <c r="F283" s="5" t="inlineStr">
         <is>
-          <t>2050</t>
+          <t>2375</t>
         </is>
       </c>
       <c r="G283" s="5" t="inlineStr">
@@ -24956,7 +24956,7 @@
       </c>
       <c r="H283" s="5" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="I283" s="5" t="inlineStr">
@@ -24966,27 +24966,27 @@
       </c>
       <c r="J283" s="5" t="inlineStr">
         <is>
-          <t>Beaubien</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K283" s="5" t="inlineStr">
         <is>
-          <t>orange</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L283" s="5" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="M283" s="5" t="inlineStr">
         <is>
-          <t>Marketplace</t>
+          <t>Centris</t>
         </is>
       </c>
       <c r="N283" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2219881575422253</t>
+          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
         </is>
       </c>
       <c r="O283" s="5" t="inlineStr">
@@ -24996,19 +24996,19 @@
       </c>
       <c r="P283" s="6" t="inlineStr">
         <is>
-          <t>Entièrement rénové, cour arrière privée, Walk Score 99, à quelques pas de cafés/restos/boulangeries/épiceries fines de la Petite-Italie, à environ 10 min du marché Jean-Talon. Lien Facebook (connexion requise)</t>
+          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
         </is>
       </c>
       <c r="Q283" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/714823210_969706739294886_222709070726311984_n.jpg?stp=c134.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=111&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=Q4rmFfALvM0Q7kNvwH2W42u&amp;_nc_oc=AdpINKj09PPc8Re8DxGgY3chRB5RnttQl9NAS-AFL9O8KTqqt1dR9NYx_1WNt0O8lww&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=JqfxygLQ7LNnSdbCmwTgsw&amp;_nc_ss=7f2a8&amp;oh=00_AQDsARrJ7YHo6O-8Zg1v5X3ykFLojfdUxVqQy1Z7t2iyQg&amp;oe=6A5DC11E</t>
+          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
         </is>
       </c>
     </row>
     <row r="284">
       <c r="A284" s="5" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B284" s="5" t="inlineStr">
@@ -25018,22 +25018,22 @@
       </c>
       <c r="C284" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 (avec sous-sol), 2 garages – Rosemont</t>
+          <t>5½ au Plateau-Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D284" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E284" s="5" t="inlineStr">
         <is>
-          <t>1889 Rue des Carrières, Montréal</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F284" s="5" t="inlineStr">
         <is>
-          <t>2375</t>
+          <t>1975</t>
         </is>
       </c>
       <c r="G284" s="5" t="inlineStr">
@@ -25043,7 +25043,7 @@
       </c>
       <c r="H284" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I284" s="5" t="inlineStr">
@@ -25068,34 +25068,34 @@
       </c>
       <c r="M284" s="5" t="inlineStr">
         <is>
-          <t>Centris</t>
+          <t>Marketplace</t>
         </is>
       </c>
       <c r="N284" s="7" t="inlineStr">
         <is>
-          <t>https://www.centris.ca/en/condos-apartments~for-rent~montreal-rosemont-la-petite-patrie/15047676</t>
+          <t>https://www.facebook.com/marketplace/item/2124372061520309</t>
         </is>
       </c>
       <c r="O284" s="5" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="P284" s="6" t="inlineStr">
         <is>
-          <t>Walk Score 94, 2 places de garage à 250$/mois chacune, rénovations récentes sous-sol et salle de bain, libre 5 jours après acceptation du bail</t>
+          <t>Annonce titre seulement, description non disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½. Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q284" s="5" t="inlineStr">
         <is>
-          <t>https://mspublic.centris.ca/media.ashx?id=ADDD250DE603764DDDDDDDDDDD&amp;t=pi&amp;w=1260&amp;h=1024&amp;sm=c</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/790150151_2283077578925626_1749367086388284890_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=ijxRbFhYaKgQ7kNvwENuJLs&amp;_nc_oc=AdqRCM7MaQD28AUVRdjZcBzo8BdTIquAZ9ZXEJ_CuW49MLQJ8m_tT8IYK6EBtN-I4h8&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=21kqsDFTPPlqY_va03ORdw&amp;_nc_ss=7f2a8&amp;oh=00_AQLzxnd4o8SoM-y6_91RzKmvUUM3My8GuhXTwpSztagGmg&amp;oe=6A9C7E28</t>
         </is>
       </c>
     </row>
     <row r="285">
       <c r="A285" s="5" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B285" s="5" t="inlineStr">
@@ -25105,7 +25105,7 @@
       </c>
       <c r="C285" s="6" t="inlineStr">
         <is>
-          <t>5½ au Plateau-Mont-Royal (Marketplace)</t>
+          <t>5½ meublé, Plateau-Mont-Royal (Marketplace), disponible 10 juin, bail minimum 1 an</t>
         </is>
       </c>
       <c r="D285" s="5" t="inlineStr">
@@ -25120,7 +25120,7 @@
       </c>
       <c r="F285" s="5" t="inlineStr">
         <is>
-          <t>1975</t>
+          <t>2100</t>
         </is>
       </c>
       <c r="G285" s="5" t="inlineStr">
@@ -25130,59 +25130,59 @@
       </c>
       <c r="H285" s="5" t="inlineStr">
         <is>
+          <t>2 (estimé)</t>
+        </is>
+      </c>
+      <c r="I285" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="J285" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="K285" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="L285" s="5" t="inlineStr">
+        <is>
+          <t>n/d</t>
+        </is>
+      </c>
+      <c r="M285" s="5" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="N285" s="7" t="inlineStr">
+        <is>
+          <t>https://www.facebook.com/marketplace/item/2129210164276639</t>
+        </is>
+      </c>
+      <c r="O285" s="5" t="inlineStr">
+        <is>
           <t>2</t>
         </is>
       </c>
-      <c r="I285" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J285" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K285" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L285" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M285" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N285" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/2124372061520309</t>
-        </is>
-      </c>
-      <c r="O285" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
       <c r="P285" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½. Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Annonce titre seulement (meublé, deux prix affichés selon la durée du bail : 2100$ et 2500$), aucune adresse ni description détaillée disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q285" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/790150151_2283077578925626_1749367086388284890_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=100&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=ijxRbFhYaKgQ7kNvwENuJLs&amp;_nc_oc=AdqRCM7MaQD28AUVRdjZcBzo8BdTIquAZ9ZXEJ_CuW49MLQJ8m_tT8IYK6EBtN-I4h8&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=21kqsDFTPPlqY_va03ORdw&amp;_nc_ss=7f2a8&amp;oh=00_AQLzxnd4o8SoM-y6_91RzKmvUUM3My8GuhXTwpSztagGmg&amp;oe=6A9C7E28</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/598654016_1589371882248064_7696909030407170199_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=N7m7nUpE6yMQ7kNvwEavU5f&amp;_nc_oc=AdoffqWsvOkDQufR2l4pvvs8I99wUIXqF-oRgpMOgZIXjIPtOiBQxSSfc9hbuhLkhtM&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=XHazkfFuptT2M_pPSTeS4Q&amp;_nc_ss=7f2a8&amp;oh=00_AQFmBd7yIIHbAZt0cYChuyEoJmxi7lgNayPM_0n-aenWnQ&amp;oe=6A9664A6</t>
         </is>
       </c>
     </row>
     <row r="286">
       <c r="A286" s="5" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B286" s="5" t="inlineStr">
@@ -25192,22 +25192,22 @@
       </c>
       <c r="C286" s="6" t="inlineStr">
         <is>
-          <t>5½ meublé, Plateau-Mont-Royal (Marketplace), disponible 10 juin, bail minimum 1 an</t>
+          <t>5 1/2 in Hochelaga (Marketplace)</t>
         </is>
       </c>
       <c r="D286" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Hochelaga-Maisonneuve</t>
         </is>
       </c>
       <c r="E286" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>n/d (secteur Hochelaga-Maisonneuve, Montréal)</t>
         </is>
       </c>
       <c r="F286" s="5" t="inlineStr">
         <is>
-          <t>2100</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G286" s="5" t="inlineStr">
@@ -25247,7 +25247,7 @@
       </c>
       <c r="N286" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2129210164276639</t>
+          <t>https://www.facebook.com/marketplace/item/2583777198803688</t>
         </is>
       </c>
       <c r="O286" s="5" t="inlineStr">
@@ -25257,19 +25257,19 @@
       </c>
       <c r="P286" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (meublé, deux prix affichés selon la durée du bail : 2100$ et 2500$), aucune adresse ni description détaillée disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Annonce titre seulement (« 5 1/2 in Hochelaga »), aucune description ni adresse disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
         </is>
       </c>
       <c r="Q286" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/598654016_1589371882248064_7696909030407170199_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=N7m7nUpE6yMQ7kNvwEavU5f&amp;_nc_oc=AdoffqWsvOkDQufR2l4pvvs8I99wUIXqF-oRgpMOgZIXjIPtOiBQxSSfc9hbuhLkhtM&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=XHazkfFuptT2M_pPSTeS4Q&amp;_nc_ss=7f2a8&amp;oh=00_AQFmBd7yIIHbAZt0cYChuyEoJmxi7lgNayPM_0n-aenWnQ&amp;oe=6A9664A6</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/764987455_1048157270911968_5209086800819479873_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=8fuDHfd2FxAQ7kNvwGWBzmX&amp;_nc_oc=AdrF-5lGt6Z8Q_hcNZtBCxKNzLwKQK14kM3UBQyfvjLyXZs14CcB6FEbpaYw4bSMoBQ&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=CInYmIZz43q5AWNfaqlZcQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHVVF-2wulz0t4MIMCVRVAytHTtSomrEGuVuullI6JrYA&amp;oe=6A790A2B</t>
         </is>
       </c>
     </row>
     <row r="287">
       <c r="A287" s="5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B287" s="5" t="inlineStr">
@@ -25279,22 +25279,22 @@
       </c>
       <c r="C287" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 in Hochelaga (Marketplace)</t>
+          <t>Appartement 5 1/2, Plateau-Mont-Royal (Marketplace)</t>
         </is>
       </c>
       <c r="D287" s="5" t="inlineStr">
         <is>
-          <t>Hochelaga-Maisonneuve</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E287" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Hochelaga-Maisonneuve, Montréal)</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F287" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>2200</t>
         </is>
       </c>
       <c r="G287" s="5" t="inlineStr">
@@ -25304,7 +25304,7 @@
       </c>
       <c r="H287" s="5" t="inlineStr">
         <is>
-          <t>2 (estimé)</t>
+          <t>2</t>
         </is>
       </c>
       <c r="I287" s="5" t="inlineStr">
@@ -25334,7 +25334,7 @@
       </c>
       <c r="N287" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2583777198803688</t>
+          <t>https://www.facebook.com/marketplace/item/1552904606229687</t>
         </is>
       </c>
       <c r="O287" s="5" t="inlineStr">
@@ -25344,19 +25344,19 @@
       </c>
       <c r="P287" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (« 5 1/2 in Hochelaga »), aucune description ni adresse disponible via le scraper. Nombre de chambres estimé à 2 selon la nomenclature standard d'un 5½, à confirmer. Lien Facebook (connexion requise) pour plus de détails.</t>
+          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
         </is>
       </c>
       <c r="Q287" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/764987455_1048157270911968_5209086800819479873_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=106&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=8fuDHfd2FxAQ7kNvwGWBzmX&amp;_nc_oc=AdrF-5lGt6Z8Q_hcNZtBCxKNzLwKQK14kM3UBQyfvjLyXZs14CcB6FEbpaYw4bSMoBQ&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=CInYmIZz43q5AWNfaqlZcQ&amp;_nc_ss=7f2a8&amp;oh=00_AQHVVF-2wulz0t4MIMCVRVAytHTtSomrEGuVuullI6JrYA&amp;oe=6A790A2B</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/720906013_1532570941905242_5666371068595538123_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=YEDvMBzBavUQ7kNvwEkVbXh&amp;_nc_oc=AdqtpC8qtzZHEdxPx9e94VcYtRcN6s4rYqZkBbexWTpuWv5UghDk5D0a0ySf9p9btAk&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=TJJlLcUljG48fNVcDPZJaA&amp;_nc_ss=7f2a8&amp;oh=00_AQBrJbOYbvchb0Tq-5jSsFppBFkZ2xgQOdjHrsx0FadLHQ&amp;oe=6A632614</t>
         </is>
       </c>
     </row>
     <row r="288">
       <c r="A288" s="5" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-17</t>
         </is>
       </c>
       <c r="B288" s="5" t="inlineStr">
@@ -25366,22 +25366,22 @@
       </c>
       <c r="C288" s="6" t="inlineStr">
         <is>
-          <t>Appartement 5 1/2, Plateau-Mont-Royal (Marketplace)</t>
+          <t>Beau 5½ à Nouveau Rosemont (Marketplace)</t>
         </is>
       </c>
       <c r="D288" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E288" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>n/d (secteur Nouveau-Rosemont, Montréal)</t>
         </is>
       </c>
       <c r="F288" s="5" t="inlineStr">
         <is>
-          <t>2200</t>
+          <t>2000</t>
         </is>
       </c>
       <c r="G288" s="5" t="inlineStr">
@@ -25421,7 +25421,7 @@
       </c>
       <c r="N288" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1552904606229687</t>
+          <t>https://www.facebook.com/marketplace/item/771126382598215</t>
         </is>
       </c>
       <c r="O288" s="5" t="inlineStr">
@@ -25431,19 +25431,19 @@
       </c>
       <c r="P288" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
+          <t>Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q288" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/720906013_1532570941905242_5666371068595538123_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=YEDvMBzBavUQ7kNvwEkVbXh&amp;_nc_oc=AdqtpC8qtzZHEdxPx9e94VcYtRcN6s4rYqZkBbexWTpuWv5UghDk5D0a0ySf9p9btAk&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=TJJlLcUljG48fNVcDPZJaA&amp;_nc_ss=7f2a8&amp;oh=00_AQBrJbOYbvchb0Tq-5jSsFppBFkZ2xgQOdjHrsx0FadLHQ&amp;oe=6A632614</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/674573089_942123441857660_1258864760862245194_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=-PqFDWdPNa8Q7kNvwG9FoYC&amp;_nc_oc=Adqy82S_lfHjbp4dkLyXqO9W2nrNBD-zKhYTIwlodmCwj46lhM9QhEG2rupuBRJOPVI&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQDV5R2cb2f6avoKzX1khDbQ_SvUKiySFkJsux9T10Rmdg&amp;oe=6A6059BA</t>
         </is>
       </c>
     </row>
     <row r="289">
       <c r="A289" s="5" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B289" s="5" t="inlineStr">
@@ -25453,7 +25453,7 @@
       </c>
       <c r="C289" s="6" t="inlineStr">
         <is>
-          <t>Beau 5½ à Nouveau Rosemont (Marketplace)</t>
+          <t>5-1/2 Rosemont (La Petite-Patrie)</t>
         </is>
       </c>
       <c r="D289" s="5" t="inlineStr">
@@ -25463,12 +25463,12 @@
       </c>
       <c r="E289" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Nouveau-Rosemont, Montréal)</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F289" s="5" t="inlineStr">
         <is>
-          <t>2000</t>
+          <t>1950</t>
         </is>
       </c>
       <c r="G289" s="5" t="inlineStr">
@@ -25508,7 +25508,7 @@
       </c>
       <c r="N289" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/771126382598215</t>
+          <t>https://www.facebook.com/marketplace/item/1249775127316090</t>
         </is>
       </c>
       <c r="O289" s="5" t="inlineStr">
@@ -25518,12 +25518,12 @@
       </c>
       <c r="P289" s="6" t="inlineStr">
         <is>
-          <t>Peu de détails disponibles dans l'annonce (pas d'adresse exacte ni de superficie). Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
         </is>
       </c>
       <c r="Q289" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/674573089_942123441857660_1258864760862245194_n.jpg?stp=c89.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=-PqFDWdPNa8Q7kNvwG9FoYC&amp;_nc_oc=Adqy82S_lfHjbp4dkLyXqO9W2nrNBD-zKhYTIwlodmCwj46lhM9QhEG2rupuBRJOPVI&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=8ft2OWSslHjx1ccZ2nFb1w&amp;_nc_ss=7f2a8&amp;oh=00_AQDV5R2cb2f6avoKzX1khDbQ_SvUKiySFkJsux9T10Rmdg&amp;oe=6A6059BA</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/671899528_1686294965723943_4545041476511987210_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xqmMQDvhJyAQ7kNvwH2BiIA&amp;_nc_oc=Adrb6HhJ7AWRb5Vln_jWCEMjozYYhefbdIyqNV0qQcHSggRpyTjrMcklU7eB9de9Y0s&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=POnFrCwMzHXIAMbS8hYJRQ&amp;_nc_ss=7f2a8&amp;oh=00_AQBeKgxbGCX6t2QjecZXjpQL0PuubZ84LadG2I8Gj_1mug&amp;oe=6A5E87C9</t>
         </is>
       </c>
     </row>
@@ -25540,7 +25540,7 @@
       </c>
       <c r="C290" s="6" t="inlineStr">
         <is>
-          <t>5-1/2 Rosemont (La Petite-Patrie)</t>
+          <t>5 1/2 lumineux à Rosemont - 2 chambres - Masson / Pie-IX</t>
         </is>
       </c>
       <c r="D290" s="5" t="inlineStr">
@@ -25550,7 +25550,7 @@
       </c>
       <c r="E290" s="5" t="inlineStr">
         <is>
-          <t>n/d (Montréal, QC)</t>
+          <t>n/d (secteur Masson / Pie-IX, Montréal)</t>
         </is>
       </c>
       <c r="F290" s="5" t="inlineStr">
@@ -25575,12 +25575,12 @@
       </c>
       <c r="J290" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>Pie-IX (mentionné dans le titre)</t>
         </is>
       </c>
       <c r="K290" s="5" t="inlineStr">
         <is>
-          <t>n/d</t>
+          <t>verte</t>
         </is>
       </c>
       <c r="L290" s="5" t="inlineStr">
@@ -25595,7 +25595,7 @@
       </c>
       <c r="N290" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/1249775127316090</t>
+          <t>https://www.facebook.com/marketplace/item/2238212030311408</t>
         </is>
       </c>
       <c r="O290" s="5" t="inlineStr">
@@ -25605,12 +25605,12 @@
       </c>
       <c r="P290" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper. Lien Facebook (connexion requise) pour plus de détails</t>
+          <t>Annonce titre seulement, description non disponible via le scraper ; secteur Masson/Pie-IX mentionné dans le titre mais distance exacte inconnue. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q290" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/671899528_1686294965723943_4545041476511987210_n.jpg?stp=c0.87.526.526a_dst-jpg_p526x395_tt6&amp;_nc_cat=109&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=xqmMQDvhJyAQ7kNvwH2BiIA&amp;_nc_oc=Adrb6HhJ7AWRb5Vln_jWCEMjozYYhefbdIyqNV0qQcHSggRpyTjrMcklU7eB9de9Y0s&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=POnFrCwMzHXIAMbS8hYJRQ&amp;_nc_ss=7f2a8&amp;oh=00_AQBeKgxbGCX6t2QjecZXjpQL0PuubZ84LadG2I8Gj_1mug&amp;oe=6A5E87C9</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/719804341_36311671888447568_3859659500532179340_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=vtlzBRqRSRoQ7kNvwHzTYPO&amp;_nc_oc=AdoFOL6FWNc1M9UybWVnYuEzJQJlAq6neF5rbnVhe9_6oLH2S29hP6IEKy2E7BpCLDg&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQB2Z-K5zeotniKSOg35MSVtER8_xPmH2m9kSVj-TPJ32A&amp;oe=6A5E8CF7</t>
         </is>
       </c>
     </row>
@@ -25627,22 +25627,22 @@
       </c>
       <c r="C291" s="6" t="inlineStr">
         <is>
-          <t>5 1/2 lumineux à Rosemont - 2 chambres - Masson / Pie-IX</t>
+          <t>Location 4 et demi Plateau, pet friendly</t>
         </is>
       </c>
       <c r="D291" s="5" t="inlineStr">
         <is>
-          <t>Rosemont-La Petite-Patrie</t>
+          <t>Le Plateau-Mont-Royal</t>
         </is>
       </c>
       <c r="E291" s="5" t="inlineStr">
         <is>
-          <t>n/d (secteur Masson / Pie-IX, Montréal)</t>
+          <t>n/d (Montréal, QC)</t>
         </is>
       </c>
       <c r="F291" s="5" t="inlineStr">
         <is>
-          <t>1950</t>
+          <t>2150</t>
         </is>
       </c>
       <c r="G291" s="5" t="inlineStr">
@@ -25662,12 +25662,12 @@
       </c>
       <c r="J291" s="5" t="inlineStr">
         <is>
-          <t>Pie-IX (mentionné dans le titre)</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="K291" s="5" t="inlineStr">
         <is>
-          <t>verte</t>
+          <t>n/d</t>
         </is>
       </c>
       <c r="L291" s="5" t="inlineStr">
@@ -25682,7 +25682,7 @@
       </c>
       <c r="N291" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/2238212030311408</t>
+          <t>https://www.facebook.com/marketplace/item/880670661257255</t>
         </is>
       </c>
       <c r="O291" s="5" t="inlineStr">
@@ -25692,12 +25692,12 @@
       </c>
       <c r="P291" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement, description non disponible via le scraper ; secteur Masson/Pie-IX mentionné dans le titre mais distance exacte inconnue. Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement (prix affiché entre 2150$ et 2350$), description non disponible via le scraper, animaux acceptés. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q291" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/719804341_36311671888447568_3859659500532179340_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=107&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=vtlzBRqRSRoQ7kNvwHzTYPO&amp;_nc_oc=AdoFOL6FWNc1M9UybWVnYuEzJQJlAq6neF5rbnVhe9_6oLH2S29hP6IEKy2E7BpCLDg&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQB2Z-K5zeotniKSOg35MSVtER8_xPmH2m9kSVj-TPJ32A&amp;oe=6A5E8CF7</t>
+          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/739200097_2136278627323814_3520943268052786943_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=gPcahdqySPYQ7kNvwGsYlqA&amp;_nc_oc=Adr3EDMhZojMTr_b6P1fzAVXVarO60w-XBK6dTJaEUmqMft4FzmSbchZ5AfV6DC3Usw&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQBgwOGHm1ihFR3tvhrAE6VDaZym-txS_aF6xIBAwy5A1Q&amp;oe=6A5EA1A8</t>
         </is>
       </c>
     </row>
@@ -25714,12 +25714,12 @@
       </c>
       <c r="C292" s="6" t="inlineStr">
         <is>
-          <t>Location 4 et demi Plateau, pet friendly</t>
+          <t>5 1/2 Rosemont avec cour privée</t>
         </is>
       </c>
       <c r="D292" s="5" t="inlineStr">
         <is>
-          <t>Le Plateau-Mont-Royal</t>
+          <t>Rosemont-La Petite-Patrie</t>
         </is>
       </c>
       <c r="E292" s="5" t="inlineStr">
@@ -25729,7 +25729,7 @@
       </c>
       <c r="F292" s="5" t="inlineStr">
         <is>
-          <t>2150</t>
+          <t>2215</t>
         </is>
       </c>
       <c r="G292" s="5" t="inlineStr">
@@ -25769,7 +25769,7 @@
       </c>
       <c r="N292" s="7" t="inlineStr">
         <is>
-          <t>https://www.facebook.com/marketplace/item/880670661257255</t>
+          <t>https://www.facebook.com/marketplace/item/1493110625829174</t>
         </is>
       </c>
       <c r="O292" s="5" t="inlineStr">
@@ -25779,104 +25779,17 @@
       </c>
       <c r="P292" s="6" t="inlineStr">
         <is>
-          <t>Annonce titre seulement (prix affiché entre 2150$ et 2350$), description non disponible via le scraper, animaux acceptés. Lien Facebook (connexion requise)</t>
+          <t>Annonce titre seulement, description non disponible via le scraper ; cour privée mentionnée. Lien Facebook (connexion requise)</t>
         </is>
       </c>
       <c r="Q292" s="5" t="inlineStr">
         <is>
-          <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t39.84726-6/739200097_2136278627323814_3520943268052786943_n.jpg?stp=c90.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=103&amp;ccb=1-7&amp;_nc_sid=92e707&amp;_nc_ohc=gPcahdqySPYQ7kNvwGsYlqA&amp;_nc_oc=Adr3EDMhZojMTr_b6P1fzAVXVarO60w-XBK6dTJaEUmqMft4FzmSbchZ5AfV6DC3Usw&amp;_nc_zt=14&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQBgwOGHm1ihFR3tvhrAE6VDaZym-txS_aF6xIBAwy5A1Q&amp;oe=6A5EA1A8</t>
-        </is>
-      </c>
-    </row>
-    <row r="293">
-      <c r="A293" s="5" t="inlineStr">
-        <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="B293" s="5" t="inlineStr">
-        <is>
-          <t>vu</t>
-        </is>
-      </c>
-      <c r="C293" s="6" t="inlineStr">
-        <is>
-          <t>5 1/2 Rosemont avec cour privée</t>
-        </is>
-      </c>
-      <c r="D293" s="5" t="inlineStr">
-        <is>
-          <t>Rosemont-La Petite-Patrie</t>
-        </is>
-      </c>
-      <c r="E293" s="5" t="inlineStr">
-        <is>
-          <t>n/d (Montréal, QC)</t>
-        </is>
-      </c>
-      <c r="F293" s="5" t="inlineStr">
-        <is>
-          <t>2215</t>
-        </is>
-      </c>
-      <c r="G293" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="H293" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I293" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="J293" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="K293" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="L293" s="5" t="inlineStr">
-        <is>
-          <t>n/d</t>
-        </is>
-      </c>
-      <c r="M293" s="5" t="inlineStr">
-        <is>
-          <t>Marketplace</t>
-        </is>
-      </c>
-      <c r="N293" s="7" t="inlineStr">
-        <is>
-          <t>https://www.facebook.com/marketplace/item/1493110625829174</t>
-        </is>
-      </c>
-      <c r="O293" s="5" t="inlineStr">
-        <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="P293" s="6" t="inlineStr">
-        <is>
-          <t>Annonce titre seulement, description non disponible via le scraper ; cour privée mentionnée. Lien Facebook (connexion requise)</t>
-        </is>
-      </c>
-      <c r="Q293" s="5" t="inlineStr">
-        <is>
           <t>https://scontent-yyz1-1.xx.fbcdn.net/v/t45.5328-4/730530074_1035539099460685_3801485303896565628_n.jpg?stp=c313.0.540.540a_dst-jpg_p180x540_tt6&amp;_nc_cat=110&amp;ccb=1-7&amp;_nc_sid=247b10&amp;_nc_ohc=_9b7saLCWEUQ7kNvwHrw_2v&amp;_nc_oc=AdoqEj5UFxI4lgfrZP0kbf8mdi_MJO6fIO-zv3fvQ5DsX656NtR6Rf8AiVxw-oho-l4&amp;_nc_zt=23&amp;_nc_ht=scontent-yyz1-1.xx&amp;_nc_gid=qCpowFOKCzme7PAXiFpzMA&amp;_nc_ss=7f2a8&amp;oh=00_AQDqhmwAH6WdMqAuOtshO7wqRdBG7RkedN25_yaUpz5ikg&amp;oe=6A5EB662</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Q293"/>
+  <autoFilter ref="A1:Q292"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N3" r:id="rId2"/>
@@ -26169,7 +26082,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N290" r:id="rId289"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N291" r:id="rId290"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N292" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="N293" r:id="rId292"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>